<commit_message>
Add project directory structure: api, user-web, admin-web
- api/: FastAPI 백엔드 초기 구조 (main, config, database, routers/services/models/utils)
- user-web/: 사용자 웹 Vue.js 초기 구조 (router, stores, views, components, locales)
- admin-web/: 관리자 웹 Vue.js 초기 구조 (동일 패턴)
- 각 폴더에 CLAUDE.md 개발 지침 템플릿 배치
- 루트 CLAUDE.md 경로/명령어 업데이트 (backend→api, frontend→user-web/admin-web)
- PLAN.md React→Vue.js 수정

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/db_specs/tpk_table_spec_20260321.xlsx
+++ b/db_specs/tpk_table_spec_20260321.xlsx
@@ -5,32 +5,34 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsshim\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\tpk_mvp\db_specs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D89B508-D2F6-45A7-BC20-8C0B9D8CE6C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{323CAD56-5039-4A7B-8423-FCD7E36D6509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="tb_user" sheetId="1" r:id="rId1"/>
-    <sheet name="tb_user_device" sheetId="2" r:id="rId2"/>
-    <sheet name="tb_exam_list" sheetId="3" r:id="rId3"/>
-    <sheet name="tb_exam_instruction" sheetId="4" r:id="rId4"/>
-    <sheet name="tb_exam_question" sheetId="5" r:id="rId5"/>
-    <sheet name="tb_exam_answer" sheetId="6" r:id="rId6"/>
-    <sheet name="tb_practice_question" sheetId="7" r:id="rId7"/>
-    <sheet name="tb_practice_answer" sheetId="8" r:id="rId8"/>
-    <sheet name="tb_question_structure" sheetId="9" r:id="rId9"/>
-    <sheet name="tb_history_exam" sheetId="10" r:id="rId10"/>
-    <sheet name="tb_history_practice" sheetId="11" r:id="rId11"/>
+    <sheet name="tb_group_code" sheetId="12" r:id="rId1"/>
+    <sheet name="tb_code" sheetId="13" r:id="rId2"/>
+    <sheet name="tb_user" sheetId="1" r:id="rId3"/>
+    <sheet name="tb_user_device" sheetId="2" r:id="rId4"/>
+    <sheet name="tb_exam_list" sheetId="3" r:id="rId5"/>
+    <sheet name="tb_exam_instruction" sheetId="4" r:id="rId6"/>
+    <sheet name="tb_exam_question" sheetId="5" r:id="rId7"/>
+    <sheet name="tb_exam_answer" sheetId="6" r:id="rId8"/>
+    <sheet name="tb_practice_question" sheetId="7" r:id="rId9"/>
+    <sheet name="tb_practice_answer" sheetId="8" r:id="rId10"/>
+    <sheet name="tb_question_structure" sheetId="9" r:id="rId11"/>
+    <sheet name="tb_history_exam" sheetId="10" r:id="rId12"/>
+    <sheet name="tb_history_practice" sheetId="11" r:id="rId13"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="145">
   <si>
     <t>tb_user : 사용자</t>
   </si>
@@ -404,6 +406,77 @@
   <si>
     <t>PK_EXAM_INSTRUCTION</t>
     <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>tb_group_code : 그룹코드</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>group_code</t>
+  </si>
+  <si>
+    <t>그룹코드</t>
+  </si>
+  <si>
+    <t>PK_GROUP_CODE</t>
+  </si>
+  <si>
+    <t>group_name</t>
+  </si>
+  <si>
+    <t>그룹코드명</t>
+  </si>
+  <si>
+    <t>group_desc</t>
+  </si>
+  <si>
+    <t>설명</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>생성시간</t>
+  </si>
+  <si>
+    <t>수정시간</t>
+  </si>
+  <si>
+    <t>tb_code : 코드</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>PK_CODE</t>
+  </si>
+  <si>
+    <t>TB_GROUP_CODE</t>
+  </si>
+  <si>
+    <t>code</t>
+  </si>
+  <si>
+    <t>코드</t>
+  </si>
+  <si>
+    <t>code_name</t>
+  </si>
+  <si>
+    <t>코드명</t>
+  </si>
+  <si>
+    <t>code_desc</t>
+  </si>
+  <si>
+    <t>코드설명</t>
+  </si>
+  <si>
+    <t>sort_order</t>
+  </si>
+  <si>
+    <t>소스순서</t>
+  </si>
+  <si>
+    <t>SMALLINT</t>
   </si>
 </sst>
 </file>
@@ -487,7 +560,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -501,6 +574,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -802,9 +876,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45C188A5-A1AF-4F10-B69D-FC35BDC4C50F}">
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -817,12 +891,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -857,17 +931,19 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>12</v>
+        <v>123</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>124</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D3" s="4">
+        <v>20</v>
+      </c>
       <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
@@ -876,24 +952,24 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>17</v>
+        <v>126</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>18</v>
+        <v>127</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="4">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>15</v>
@@ -905,18 +981,18 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>20</v>
+        <v>128</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>21</v>
+        <v>129</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D5" s="4">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="3"/>
@@ -926,45 +1002,47 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D6" s="4">
-        <v>20</v>
-      </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>130</v>
+      </c>
       <c r="G6" s="4"/>
       <c r="H6" s="3"/>
       <c r="I6" s="4"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>25</v>
+        <v>131</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="4">
-        <v>1</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D7" s="4"/>
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="3"/>
@@ -972,22 +1050,24 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D8" s="4">
+        <v>50</v>
+      </c>
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="3"/>
@@ -995,24 +1075,22 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>32</v>
+        <v>132</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="4">
-        <v>50</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="3"/>
@@ -1020,53 +1098,30 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D10" s="4">
+        <v>50</v>
+      </c>
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="3"/>
       <c r="I10" s="4"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="4">
-        <v>50</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -1075,9 +1130,243 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="5" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
+    <col min="9" max="9" width="5" customWidth="1"/>
+    <col min="10" max="10" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A4" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="4"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="4">
+        <v>50</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="4"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="4"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="4">
+        <v>50</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="4"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -1090,12 +1379,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1130,12 +1419,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>14</v>
@@ -1149,170 +1438,160 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>12</v>
+        <v>95</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>96</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4" t="s">
-        <v>15</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="D4" s="4">
+        <v>50</v>
+      </c>
+      <c r="E4" s="4"/>
       <c r="F4" s="3"/>
       <c r="G4" s="4"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I4" s="4"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>53</v>
+        <v>97</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>54</v>
+        <v>98</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="D5" s="4"/>
-      <c r="E5" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="E5" s="4"/>
       <c r="F5" s="3"/>
       <c r="G5" s="4"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I5" s="4"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>68</v>
+        <v>99</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="D6" s="4"/>
-      <c r="E6" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="E6" s="4"/>
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I6" s="4"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>105</v>
+        <v>24</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>106</v>
+        <v>25</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="4">
-        <v>20</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G7" s="4"/>
       <c r="H7" s="3"/>
       <c r="I7" s="4"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>107</v>
+        <v>27</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>108</v>
+        <v>28</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="3"/>
+      <c r="E8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="G8" s="4"/>
       <c r="H8" s="3"/>
       <c r="I8" s="4"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>109</v>
+        <v>31</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>110</v>
+        <v>32</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="3"/>
+        <v>19</v>
+      </c>
+      <c r="D9" s="4">
+        <v>50</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>33</v>
+      </c>
       <c r="G9" s="4"/>
       <c r="H9" s="3"/>
       <c r="I9" s="4"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="4">
-        <v>1</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="3"/>
@@ -1320,101 +1599,30 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D11" s="4">
+        <v>50</v>
+      </c>
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="3"/>
       <c r="I11" s="4"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="4">
-        <v>50</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G12" s="4"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13" s="4"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="4">
-        <v>50</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G14" s="4"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -1422,10 +1630,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -1438,12 +1646,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1478,7 +1686,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>102</v>
       </c>
@@ -1497,13 +1705,13 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -1530,12 +1738,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>39</v>
@@ -1551,44 +1759,52 @@
         <v>15</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="K5" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A6" s="3" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>105</v>
-      </c>
       <c r="B6" s="3" t="s">
-        <v>106</v>
+        <v>69</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="4">
-        <v>20</v>
-      </c>
-      <c r="E6" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D7" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D7" s="4">
+        <v>20</v>
+      </c>
       <c r="E7" s="4"/>
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
@@ -1597,15 +1813,15 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -1616,47 +1832,43 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>25</v>
+        <v>110</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="4">
-        <v>1</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>26</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="3"/>
       <c r="G9" s="4"/>
       <c r="H9" s="3"/>
       <c r="I9" s="4"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1</v>
+      </c>
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="3"/>
@@ -1664,24 +1876,22 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="4">
-        <v>50</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D11" s="4"/>
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="3"/>
@@ -1689,22 +1899,24 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D12" s="4">
+        <v>50</v>
+      </c>
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="3"/>
@@ -1712,30 +1924,53 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D13" s="4">
-        <v>50</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D13" s="4"/>
       <c r="E13" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="3"/>
       <c r="I13" s="4"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="4">
+        <v>50</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G14" s="4"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -1743,10 +1978,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -1759,12 +1994,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1799,15 +2034,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>103</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
@@ -1818,76 +2053,78 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="K3" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>42</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="3"/>
-      <c r="G4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G4" s="4"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="4">
-        <v>20</v>
-      </c>
-      <c r="E5" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="F5" s="3"/>
       <c r="G5" s="4"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>46</v>
+        <v>105</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>47</v>
+        <v>106</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D6" s="4">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="3"/>
@@ -1897,19 +2134,17 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>48</v>
+        <v>107</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>49</v>
+        <v>108</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="4">
-        <v>20</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
@@ -1918,19 +2153,17 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>50</v>
+        <v>109</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>51</v>
+        <v>110</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="4">
-        <v>20</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="3"/>
       <c r="G8" s="4"/>
@@ -1939,7 +2172,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
@@ -1964,7 +2197,7 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>27</v>
       </c>
@@ -1987,7 +2220,7 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>31</v>
       </c>
@@ -2012,7 +2245,7 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>34</v>
       </c>
@@ -2035,7 +2268,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>36</v>
       </c>
@@ -2059,6 +2292,310 @@
       <c r="I13" s="4"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC3182D5-E992-4F10-9BA9-EA3D1063629B}">
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="5" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
+    <col min="9" max="9" width="4.75" customWidth="1"/>
+    <col min="10" max="11" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A3" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="4">
+        <v>20</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A4" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A5" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="4">
+        <v>50</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A6" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="4">
+        <v>200</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A7" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="4">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="4"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" s="4"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="4">
+        <v>50</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="4"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A12" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="5">
+        <v>50</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -2067,9 +2604,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -2082,12 +2619,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2122,12 +2659,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>14</v>
@@ -2141,24 +2678,24 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="4">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>15</v>
@@ -2170,17 +2707,19 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D5" s="4">
+        <v>100</v>
+      </c>
       <c r="E5" s="4"/>
       <c r="F5" s="3"/>
       <c r="G5" s="4"/>
@@ -2189,18 +2728,18 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D6" s="4">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="3"/>
@@ -2210,7 +2749,7 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>24</v>
       </c>
@@ -2235,7 +2774,7 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>27</v>
       </c>
@@ -2258,7 +2797,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>31</v>
       </c>
@@ -2283,7 +2822,7 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>34</v>
       </c>
@@ -2306,7 +2845,7 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>36</v>
       </c>
@@ -2338,9 +2877,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:K10"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -2353,12 +2892,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2393,12 +2932,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>39</v>
@@ -2412,27 +2951,27 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>121</v>
+        <v>40</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4" t="s">
@@ -2443,23 +2982,25 @@
         <v>15</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>121</v>
+        <v>40</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D5" s="4">
+        <v>20</v>
+      </c>
       <c r="E5" s="4"/>
       <c r="F5" s="3"/>
       <c r="G5" s="4"/>
@@ -2468,95 +3009,87 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D6" s="4">
-        <v>1</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>26</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="3"/>
       <c r="G6" s="4"/>
       <c r="H6" s="3"/>
       <c r="I6" s="4"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>30</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="D7" s="4">
+        <v>20</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="3"/>
       <c r="G7" s="4"/>
       <c r="H7" s="3"/>
       <c r="I7" s="4"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D8" s="4">
-        <v>50</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>33</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="3"/>
       <c r="G8" s="4"/>
       <c r="H8" s="3"/>
       <c r="I8" s="4"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="3"/>
@@ -2564,30 +3097,101 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="4">
-        <v>50</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="3"/>
       <c r="I10" s="4"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="4">
+        <v>50</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="4"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A13" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="4">
+        <v>50</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -2596,9 +3200,9 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -2611,12 +3215,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2651,7 +3255,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>53</v>
       </c>
@@ -2659,7 +3263,7 @@
         <v>54</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
@@ -2670,56 +3274,46 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>113</v>
+        <v>56</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D4" s="4">
+        <v>20</v>
+      </c>
       <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="3"/>
-      <c r="G4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>120</v>
-      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="3"/>
       <c r="I4" s="4"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="4">
-        <v>20</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="3"/>
       <c r="G5" s="4"/>
@@ -2728,18 +3322,18 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D6" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="3"/>
@@ -2749,206 +3343,126 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>74</v>
+        <v>24</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="4">
-        <v>20</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="G7" s="4"/>
       <c r="H7" s="3"/>
       <c r="I7" s="4"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="3"/>
+      <c r="E8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="G8" s="4"/>
       <c r="H8" s="3"/>
       <c r="I8" s="4"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>77</v>
+        <v>32</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="3"/>
+        <v>19</v>
+      </c>
+      <c r="D9" s="4">
+        <v>50</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>33</v>
+      </c>
       <c r="G9" s="4"/>
       <c r="H9" s="3"/>
       <c r="I9" s="4"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="4">
-        <v>10</v>
-      </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="3"/>
+        <v>29</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="G10" s="4"/>
       <c r="H10" s="3"/>
       <c r="I10" s="4"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="4">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="3"/>
       <c r="I11" s="4"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G12" s="4"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D13" s="4">
-        <v>50</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G13" s="4"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G14" s="4"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="4">
-        <v>50</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G15" s="4"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -2957,9 +3471,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K10"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -2972,12 +3486,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -3012,7 +3526,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>53</v>
       </c>
@@ -3031,24 +3545,24 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>118</v>
+        <v>62</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>39</v>
@@ -3062,24 +3576,18 @@
         <v>15</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>67</v>
@@ -3093,7 +3601,7 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>24</v>
       </c>
@@ -3118,7 +3626,7 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>27</v>
       </c>
@@ -3141,7 +3649,7 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>31</v>
       </c>
@@ -3166,7 +3674,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>34</v>
       </c>
@@ -3189,7 +3697,7 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>36</v>
       </c>
@@ -3221,9 +3729,9 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -3236,12 +3744,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -3276,15 +3784,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
@@ -3295,39 +3803,49 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>70</v>
+        <v>113</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="4">
-        <v>20</v>
-      </c>
-      <c r="E4" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="F4" s="3"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="3"/>
+      <c r="G4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="I4" s="4"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>19</v>
@@ -3343,12 +3861,12 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>19</v>
@@ -3364,17 +3882,19 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D7" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D7" s="4">
+        <v>20</v>
+      </c>
       <c r="E7" s="4"/>
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
@@ -3383,15 +3903,15 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -3402,19 +3922,17 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="4">
-        <v>10</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="3"/>
       <c r="G9" s="4"/>
@@ -3423,30 +3941,28 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D10" s="4">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E10" s="4"/>
-      <c r="F10" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="F10" s="3"/>
       <c r="G10" s="4"/>
       <c r="H10" s="3"/>
       <c r="I10" s="4"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>24</v>
       </c>
@@ -3471,7 +3987,7 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>27</v>
       </c>
@@ -3494,7 +4010,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>31</v>
       </c>
@@ -3519,7 +4035,7 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
         <v>34</v>
       </c>
@@ -3542,7 +4058,7 @@
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
         <v>36</v>
       </c>
@@ -3574,9 +4090,9 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -3589,12 +4105,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -3629,12 +4145,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>39</v>
@@ -3648,78 +4164,86 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>89</v>
+        <v>119</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="K3" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A4" s="3" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="B4" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A5" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="4">
-        <v>1</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="3"/>
       <c r="G5" s="4"/>
       <c r="H5" s="3"/>
       <c r="I5" s="4"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1</v>
+      </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="3"/>
@@ -3727,24 +4251,22 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="4">
-        <v>50</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D7" s="4"/>
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="3"/>
@@ -3752,22 +4274,24 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D8" s="4">
+        <v>50</v>
+      </c>
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="3"/>
@@ -3775,30 +4299,53 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="4">
-        <v>50</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="3"/>
       <c r="I9" s="4"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A10" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="4">
+        <v>50</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="4"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -3807,9 +4354,9 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -3822,12 +4369,12 @@
     <col min="10" max="11" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="17.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -3862,12 +4409,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>14</v>
@@ -3881,24 +4428,24 @@
         <v>15</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="4">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="3"/>
@@ -3908,17 +4455,19 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D5" s="4">
+        <v>20</v>
+      </c>
       <c r="E5" s="4"/>
       <c r="F5" s="3"/>
       <c r="G5" s="4"/>
@@ -3927,17 +4476,19 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>99</v>
+        <v>74</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D6" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="D6" s="4">
+        <v>20</v>
+      </c>
       <c r="E6" s="4"/>
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
@@ -3946,95 +4497,81 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>24</v>
+        <v>78</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="4">
-        <v>1</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>26</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="3"/>
       <c r="G7" s="4"/>
       <c r="H7" s="3"/>
       <c r="I7" s="4"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>27</v>
+        <v>76</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D8" s="4"/>
-      <c r="E8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>30</v>
-      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="3"/>
       <c r="G8" s="4"/>
       <c r="H8" s="3"/>
       <c r="I8" s="4"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
-        <v>31</v>
+        <v>80</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D9" s="4">
-        <v>50</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>33</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="3"/>
       <c r="G9" s="4"/>
       <c r="H9" s="3"/>
       <c r="I9" s="4"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
-        <v>34</v>
+        <v>86</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4" t="s">
-        <v>15</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4"/>
       <c r="F10" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="3"/>
@@ -4042,24 +4579,24 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="4">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="3"/>
@@ -4067,6 +4604,102 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="4">
+        <v>50</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G14" s="4"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="4">
+        <v>50</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G15" s="4"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>